<commit_message>
Adjust prompt to prevent flakiness in eval judge
</commit_message>
<xml_diff>
--- a/skills/skill-test/example/brain-tumor-age-distribution-only.xlsx
+++ b/skills/skill-test/example/brain-tumor-age-distribution-only.xlsx
@@ -457,12 +457,12 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>/ccdi-federation-ai-copilot
-Using sample-diagnosis metadata, show the age distribution of brain-tumor patients across the CCDI Data Federation. Deduplicate to patients where possible and report how many records have known age vs missing age.</t>
+Using sample-diagnosis metadata with search=brain only (do not expand into other diagnosis terms, diagnosis_category PV lists, or phrase variants like "brain tumor"), show the age distribution of brain-tumor patients across the CCDI Data Federation. Deduplicate to patients where possible and report how many records have known age vs missing age.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GET /sample-diagnosis; age bins; known vs missing age coverage (~263 known). Known age records ~263 (±10%).</t>
+          <t>GET /sample-diagnosis?search=brain; age bins; known vs missing age coverage (~263 known). Must use search=brain only — not other diagnosis terms or PV lists. Known age records ~263 (±10%).</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>